<commit_message>
feat(ui): integrazione redesign PMA (pma-theme, layout, admin, ECG Cloudinary, dashboard centrale)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Prompt/Modifiche da fare.xlsx
+++ b/Prompt/Modifiche da fare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_mie\PMApp\Prompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F859F543-E15D-441C-8A54-991DD4564DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9FD15B-5C72-40CD-87D8-788D6BEE44B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Elenco" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="104">
   <si>
     <t>Descrizione</t>
   </si>
@@ -51,15 +51,6 @@
     <t>FATTO</t>
   </si>
   <si>
-    <t>Modifica testo breve con tipo evento e dettagli evento</t>
-  </si>
-  <si>
-    <t>Viste mobile</t>
-  </si>
-  <si>
-    <t>V2</t>
-  </si>
-  <si>
     <t>Campo</t>
   </si>
   <si>
@@ -126,9 +117,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Non carica firma medico</t>
-  </si>
-  <si>
     <t>CUTE</t>
   </si>
   <si>
@@ -315,53 +303,6 @@
     <t>ALTRO &gt;EO</t>
   </si>
   <si>
-    <t>Problema scrittura data di nascita</t>
-  </si>
-  <si>
-    <t>Farmaco da elenco/manuale: non si può fare che se farmaco non è in elenco lo crea dallo stesso menu? Altrimenti se proprio non si riesce almeno creare pulsante "da elenco" o "manuale" ma così dai per scontato che chi scrive sappia a memoria tutti i farmaci disponibili...</t>
-  </si>
-  <si>
-    <t>Creare elenco farmaci usati</t>
-  </si>
-  <si>
-    <t>V3</t>
-  </si>
-  <si>
-    <t>V4</t>
-  </si>
-  <si>
-    <t>Campi per EO veloce da impostare in impostazioni</t>
-  </si>
-  <si>
-    <t>La prima volta che un operatore fa login non vede tutti i pazienti del PMA ma deve cliccare su "dashboard PMA" per farli caricare. Ho notato che ci sono due root diverse chiamate tutte "Dashboard PMA", una si chiama /PMA_lecco e una /esempio</t>
-  </si>
-  <si>
-    <t>Perché se con CENTRALE clicco su "Dashboard manifestazione" mi dice "evento non trovato"?. Il pulsante "DASHBOARD" sotto "MANIFESTAZIONE" serve alla centrale per vedere lo stato dei PMA. Vede un elenco dei PMA dell'evento. Per ogni PMA vede: pazienti in arrivo, in attesa, in carico, suddivisi per codice colore. 
-Inoltre ha pulsante "RICERCA" per cercare pazienti dimessi.
-Vede un contatore che somma i pazienti "IN CARICO" mostrando accanto il numero dei posti letto di quel PMA. Se numero "IN CARICO" &lt;50% colore verde, se &gt;50% colore giallo, se &gt;75% colore rosso.</t>
-  </si>
-  <si>
-    <t>Dashboard PMA deve mostrare solo la dashboard del PMA a cui il personale è associato per il rank MEDICO, INFERMIERE, SOCCORRITORE, TRIAGE</t>
-  </si>
-  <si>
-    <t>Cercare pazienti per pettorale</t>
-  </si>
-  <si>
-    <t>Scansione tessera sanitaria</t>
-  </si>
-  <si>
-    <t>Controllare PV default</t>
-  </si>
-  <si>
-    <t>Cambio UI PMA</t>
-  </si>
-  <si>
-    <t>Campi separati per telefono e mail</t>
-  </si>
-  <si>
-    <t>Firma paziente non scrive</t>
-  </si>
-  <si>
     <t>Rank</t>
   </si>
   <si>
@@ -378,6 +319,27 @@
   </si>
   <si>
     <t>Triage</t>
+  </si>
+  <si>
+    <t>v5</t>
+  </si>
+  <si>
+    <t>Firma paziente e firma medico non vengono messe nel PDF</t>
+  </si>
+  <si>
+    <t>I pazienti "In arrivo" dalla vista PMA si possono aprire solo cliccando su una barretta. Crea un campo che avvolga il nome completamente cliccabile per aprire la scheda paziente.</t>
+  </si>
+  <si>
+    <t>I pazienti creati da RANK CENTRALE hanno tutti tipo "Trasportato"</t>
+  </si>
+  <si>
+    <t>Se paziente creato da RANK CENTRALE sotto il campo "TRASPORTATO DA" crea un campo per selezionare il PMA di destinazione a cui mandare il paziente. Se un solo PMA allora è impostato quello di default.</t>
+  </si>
+  <si>
+    <t>Crea una notifica PUSH quando la centrale crea un paziente destinato a quel PMA, attivata da un pulsante "ALLERTA PMA" in fondo al tab GENERALE della scheda paziente. Il pulsante è visibile e cliccabile solo se RANK è CENTRALE:</t>
+  </si>
+  <si>
+    <t>Sistemare dimensione UI</t>
   </si>
 </sst>
 </file>
@@ -723,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
@@ -742,32 +704,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>100</v>
       </c>
@@ -775,138 +734,28 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
+    <row r="5" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
       <c r="B7" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="195" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -963,673 +812,673 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22F5A09E-F43C-4C61-819D-8CF580A11651}">
   <dimension ref="A1:C82"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="43.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B57" s="1" t="s">
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B58" s="1" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B59" s="1" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B60" s="1" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B61" s="1" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B62" s="1" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B63" s="1" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B64" s="1" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B65" s="1" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B66" s="1" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B67" s="1" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B68" s="1" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B69" s="1" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B70" s="1" t="s">
+      <c r="B74" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B71" s="1" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B76" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B72" s="1" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B77" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B78" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B74" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B75" s="1" t="s">
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A76" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B76" s="1" t="s">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A77" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B77" s="1" t="s">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A79" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A80" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A81" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1648,32 +1497,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI: chip neutri allineati alle pill codice colore; flussi PMA e manifestazione
- Chip globali e pma-action-chip: stessa scala .pma-pill (variabili tema), colori Bianco off
- Esclusioni pma-theme-skip per menu, overlay e pulsanti solo icona
- Partecipanti Excel, redirect post-login, prestazioni PDF/cartella, vercel.json SPA
- Varie pagine manifestazione, PMA dashboard, scheda paziente e admin

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Prompt/Modifiche da fare.xlsx
+++ b/Prompt/Modifiche da fare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_mie\PMApp\Prompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9FD15B-5C72-40CD-87D8-788D6BEE44B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46988EA5-AB1D-4189-9E63-0943E167A9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="129">
   <si>
     <t>Descrizione</t>
   </si>
@@ -340,6 +340,81 @@
   </si>
   <si>
     <t>Sistemare dimensione UI</t>
+  </si>
+  <si>
+    <t>Solo l'utente MEDICO può impostare lo stato su "DIMESSO". Elimina lo stato "ERRORE". Se non riesci a capire che stato mettere crea uno stato "IN SOSPESO". Togli agli altri RANK (a parte Superadmin) la possibilità di accedere a qualsiasi pulsante che metta lo imposti paziente su "DIMESSO".</t>
+  </si>
+  <si>
+    <t>Da DASHBOARD centrale elimina "ultimi 10 dimessi per PMA"</t>
+  </si>
+  <si>
+    <t>PMA -&gt; lista pazienti in carico -&gt; fai in modo che un paziente si possa aprire cliccando su tutta la sua "riga" non solament sul nome. Allo stesso modo in "pazienti in arrivo" deve essere facile da cliccare.</t>
+  </si>
+  <si>
+    <t>PAZIENTI IN ARRIVO -&gt; visibili e modificabili da tutti. Lo stato "IN ARRIVO" può essere impostato solamente da RANK centrale. Tutti gli altri utenti non lo possono impsotare. Per ogni paziente "IN ARRIVO" crea però un pulsante "PRENDI IN CARICO" (accessibile a MEDICO, INFERMIERE, SOCCORRITORE, TRIAGE) che cambia lo stato "IN CARICO". Inoltre un paziente "IN ARRIVO" non deve rientrare nella conta dei pazienti che occupano i posti letto del PMA. Ad es: 4 pz in carico e 2 in arrivo. I pazienti che occupano posti letto sono solo 4.</t>
+  </si>
+  <si>
+    <t>In impostazioni PMA crea un campo apposta per i farmaci usati chiamandolo "Elenco farmaci usati"</t>
+  </si>
+  <si>
+    <t>Il pulsante "PRENDI IN CARICO" per i pazienti in arrivo deve essere molto piccolo e sulla stessa riga del nome paziente per occupare poco spazio</t>
+  </si>
+  <si>
+    <t>Elimina da "STATO" nella scheda paziente il pulsante "DIMESSO" per settare lo stato su DIMESSO per tutti gli utenti. Lo stato "DIMESSO" può essere settato solamente con il comando "DIMETTI PAZIENTE" In Tab dimissioni se RANK è medico.</t>
+  </si>
+  <si>
+    <t>Se RANK è centrale quando apre la vista PMA tutto gli deve comparire in SOLA LETTURA</t>
+  </si>
+  <si>
+    <t>Nel PDF generato sezione "EO RAPIDO" puoi mettere le varie categorie con le voci flaggate in colonne anziché come un testo di fila? Come se fosse una tabella con GENERALE, NEUROLOGICO, etc…. Con sotto tutti i valori</t>
+  </si>
+  <si>
+    <t>Nel PDF generato affianca firma paziente e medico per risparmiare spazio</t>
+  </si>
+  <si>
+    <t>Nell'elenco pazienti dimessi se RANK è MEDICO crea un pulsante "RIPRENDI IN CARICO" che ri-apre il paziente settandone lo stato nuovamente "IN CARICO". In "GENERALI" deve comparire un timestamp con data e ora di ripresa in carico.</t>
+  </si>
+  <si>
+    <t>In dimissione dopo NOTE DIMISSIONE inserisci due testi che sono CONSENSO GENERICO ALLE CURE e CONSENSO PRIVACY il cui valore viene inserito in due caselle di testo dedicate in "IMPOSTAZIONI MANIFESTAZIONE"</t>
+  </si>
+  <si>
+    <t>Se esito è "RIFIUTA INVIO IN PS" fai comparire un terzo testo che si chiama "RIFIUTO INVIO IN PS" il cui valore viene inserito analogamente ai due campi appena creati in "IMPOSTAZIONI MANIFESTAZIONE"</t>
+  </si>
+  <si>
+    <t>In "IMPOSTAZIONI MANIFESTAZIONE" permettimi di creare dei "PRESET DIMISSIONE" che il medico può importare, anche più di uno, mentre compila le NOTE DIMISSIONE</t>
+  </si>
+  <si>
+    <t>Inserisci i testi consenso e se presente il testo "RIFIUTO INVIO IN PS" nel PDF</t>
+  </si>
+  <si>
+    <t>Sposta i campi per impostare questi tre testi in fondo a "IMPOSTAZIONI"</t>
+  </si>
+  <si>
+    <t>Avendo cambiato il colore della barra in alto non si vedono più i testi dei contatori con i codici colori, scrivili in bianco.</t>
+  </si>
+  <si>
+    <t>Nella scheda paziente crea un piccolo tasto "ALLEGA ECG" con il simbolo di un elettrocardiogramma che permetta di allegare una foto dell'ECG del paziente da caricare allegata alla scheda, il file finisce su cloudinary. Metti il tasto sulla stessa riga di "PRESTAZIONI" per risparmiare spazio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DASHBOARD CENTRALE: elimina la riga scorrevole "ULTIMI EVENTI-DIMESSI". </t>
+  </si>
+  <si>
+    <t>DASHBOARD CENTRALE: in "VISTA RAPIDA PMA" sotto carico operativo - logistica - creazione rapida crea due colonne che mostrano la lista dei pz in carico e degli ultimi 5 pz dimessi. Accanto al tasto "APRI DASHBOARD PMA" poi aggiungi il pulsante "PAZIENTI DIMESSI" esattamente uguale al medesimo nella DASHBOARD PMA</t>
+  </si>
+  <si>
+    <t>DASHBOARD CENTRALE: comprimi la parte "ricerca dimessi", apribile solo se si clicca sopra</t>
+  </si>
+  <si>
+    <t>DASHBOARD PMA: togli i pulsanti in basso e lascia solo quelli in alto</t>
+  </si>
+  <si>
+    <t>RANK centrale deve poter leggere, modificare, creare e cancellare "CODICI MINORI" che ora è disabilitato nella vista PMA. Abilitalo.</t>
+  </si>
+  <si>
+    <t>RANK centrale deve poter leggere, modificare, creare e cancellare utenti in automatico legati alla stessa manifestazione, assegnandoli al PMA. Quindi se crea un utente questo di default è legato a quella manifestazione. Quindi deve pote aprire dal menu elenco utenti.</t>
+  </si>
+  <si>
+    <t>Per ogni utente aggiungi i campi facoltativi: numero di telefono, email, note. Rendi "nome" obbligatorio. Se hanno numero di telefono agisci in background copiando il contatto in "rubrica" di quella manifestazione compilando le celle nome e numero e "note" solo se compilata</t>
   </si>
 </sst>
 </file>
@@ -393,7 +468,67 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -411,11 +546,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B8A6B443-A6A4-4AC4-9B35-145579C78896}" name="Tabella1" displayName="Tabella1" ref="A1:C17" insertRowShift="1" totalsRowShown="0">
-  <autoFilter ref="A1:C17" xr:uid="{B8A6B443-A6A4-4AC4-9B35-145579C78896}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B8A6B443-A6A4-4AC4-9B35-145579C78896}" name="Tabella1" displayName="Tabella1" ref="A1:C32" insertRowShift="1" totalsRowShown="0">
+  <autoFilter ref="A1:C32" xr:uid="{B8A6B443-A6A4-4AC4-9B35-145579C78896}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5968C67A-E4F2-4B64-976F-B0E15A919F5A}" name="Ver"/>
-    <tableColumn id="2" xr3:uid="{ECAC3DA7-D7A8-4482-9EF6-5C441AD18BFC}" name="Descrizione" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{ECAC3DA7-D7A8-4482-9EF6-5C441AD18BFC}" name="Descrizione" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{BF548B9B-4356-4258-A960-94DD9A1EA8C4}" name="Stato"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -685,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
@@ -739,7 +874,7 @@
         <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -758,8 +893,213 @@
         <v>3</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="165" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="105" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B31" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="A2:C2">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"""IN CORSO"""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>